<commit_message>
[refs #36200] List of projects and activities formatting.
- Column B width (Agency): Set the width of Column B to match Column C (ODP), so both columns have equal width.
- Project title (wrapping/top alignment): Enable text wrapping on the project title column and top-align values.
- Top alignment values: Set top alignment for values in columns Agency, ODP, and CO2.
- Remove zero values: Where a cell value is 0, display blank instead of "0".
- Column D font size: Set font size of Column D to 11 (Currently size 10).
- Agency row alignment: Right-align text in agency rows.
- Country total rows (merge and right-align): For rows with “Total for country X”, merge Columns A and B into a single cell and right-align text.
- Country total label casing: Convert country totals from uppercase to normal case. Example: "Total for ANGOLA" → "Total for Angola".
</commit_message>
<xml_diff>
--- a/core/api/export/templates/blanket_approval_details_template.xlsx
+++ b/core/api/export/templates/blanket_approval_details_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/david/Work/edw/ors-multilateralfund/core/api/export/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{288AC9A1-909E-764E-9007-253A0A133B62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{564EB7E8-7876-8A47-80FF-1F0C29E2BAA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2100" yWindow="1560" windowWidth="26420" windowHeight="16660" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -192,11 +192,8 @@
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -253,6 +250,24 @@
     </xf>
     <xf numFmtId="3" fontId="3" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -453,159 +468,158 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="58.5" customWidth="1"/>
-    <col min="2" max="2" width="22.5" customWidth="1"/>
-    <col min="3" max="3" width="13.33203125" customWidth="1"/>
-    <col min="4" max="4" width="10.1640625" customWidth="1"/>
+    <col min="2" max="4" width="10.1640625" customWidth="1"/>
     <col min="5" max="5" width="10.5" customWidth="1"/>
     <col min="6" max="6" width="11.1640625" customWidth="1"/>
     <col min="7" max="7" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" s="2"/>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
+    <row r="1" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
     </row>
     <row r="2" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="3" t="s">
+      <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" s="5"/>
-      <c r="B3" s="5"/>
-      <c r="C3" s="6" t="s">
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+    </row>
+    <row r="3" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="4"/>
+      <c r="B3" s="4"/>
+      <c r="C3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="G3" s="6" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="8"/>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
+      <c r="B4" s="7"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="2"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="12"/>
-      <c r="G6" s="12"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" s="20" t="s">
+      <c r="A7" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="13">
-        <v>0</v>
-      </c>
-      <c r="D7" s="11"/>
-      <c r="E7" s="21">
-        <v>0</v>
-      </c>
-      <c r="F7" s="21">
-        <v>0</v>
-      </c>
-      <c r="G7" s="22">
+      <c r="C7" s="25">
+        <v>0</v>
+      </c>
+      <c r="D7" s="25"/>
+      <c r="E7" s="20">
+        <v>0</v>
+      </c>
+      <c r="F7" s="20">
+        <v>0</v>
+      </c>
+      <c r="G7" s="21">
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="2"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="15"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="12"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" s="16"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="15"/>
+      <c r="A9" s="15"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="12"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10" s="8"/>
-      <c r="B10" s="8" t="s">
+      <c r="A10" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="17">
-        <v>0</v>
-      </c>
-      <c r="D10" s="17">
-        <v>0</v>
-      </c>
-      <c r="E10" s="23">
-        <v>0</v>
-      </c>
-      <c r="F10" s="23">
-        <v>0</v>
-      </c>
-      <c r="G10" s="24">
+      <c r="B10" s="28"/>
+      <c r="C10" s="16">
+        <v>0</v>
+      </c>
+      <c r="D10" s="16">
+        <v>0</v>
+      </c>
+      <c r="E10" s="22">
+        <v>0</v>
+      </c>
+      <c r="F10" s="22">
+        <v>0</v>
+      </c>
+      <c r="G10" s="23">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="E2:G2"/>
+    <mergeCell ref="A10:B10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
[refs #36200] DB export changes.
## Approval summary

- only include v3 projects for submission_status == "approved"
- Approval summary: insert extra row on top (start at row 2)

## Summary of projects:

- Add one row at the top (table should start at row 2)
- Adjust column character widths: Column A = "36", Column B and C ="8", Column D and E ="14"
- Column E shift "(US$)" below "principle", did the same for "amounts_recommended" column.
- Merge Column A and B for Total row
- Make entire Total row bold
- Add borders to all cells in table

## List of projects and activities (blanket approval)

- Add one row at the top(table should start at row 3)
- Wrap text in column A -- now enforced in python
</commit_message>
<xml_diff>
--- a/core/api/export/templates/blanket_approval_details_template.xlsx
+++ b/core/api/export/templates/blanket_approval_details_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/david/Work/edw/ors-multilateralfund/core/api/export/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{564EB7E8-7876-8A47-80FF-1F0C29E2BAA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ECBEFA7-2DE5-6347-A289-D7D39E84480B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2100" yWindow="1560" windowWidth="26420" windowHeight="16660" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -251,23 +251,23 @@
     <xf numFmtId="3" fontId="3" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -464,7 +464,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A2:G11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="58.5" customWidth="1"/>
@@ -474,78 +474,67 @@
     <col min="7" max="7" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-    </row>
-    <row r="2" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="29" t="s">
+    <row r="2" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+    </row>
+    <row r="3" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="24" t="s">
+      <c r="E3" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-    </row>
-    <row r="3" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="5" t="s">
+      <c r="F3" s="28"/>
+      <c r="G3" s="28"/>
+    </row>
+    <row r="4" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="4"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E4" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F4" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G4" s="6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" s="26" t="s">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="7"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="9"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" s="18" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="1"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
+      <c r="B5" s="7"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="18" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="10"/>
@@ -555,39 +544,41 @@
       <c r="G6" s="11"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="1"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="27" t="s">
+      <c r="B8" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="25">
-        <v>0</v>
-      </c>
-      <c r="D7" s="25"/>
-      <c r="E7" s="20">
-        <v>0</v>
-      </c>
-      <c r="F7" s="20">
-        <v>0</v>
-      </c>
-      <c r="G7" s="21">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8" s="17" t="s">
+      <c r="C8" s="24">
+        <v>0</v>
+      </c>
+      <c r="D8" s="24"/>
+      <c r="E8" s="20">
+        <v>0</v>
+      </c>
+      <c r="F8" s="20">
+        <v>0</v>
+      </c>
+      <c r="G8" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="1"/>
-      <c r="C8" s="12"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="13"/>
-      <c r="F8" s="13"/>
-      <c r="G8" s="14"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" s="15"/>
       <c r="B9" s="1"/>
       <c r="C9" s="12"/>
       <c r="D9" s="10"/>
@@ -596,30 +587,39 @@
       <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10" s="28" t="s">
+      <c r="A10" s="15"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="12"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="14"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="28"/>
-      <c r="C10" s="16">
-        <v>0</v>
-      </c>
-      <c r="D10" s="16">
-        <v>0</v>
-      </c>
-      <c r="E10" s="22">
-        <v>0</v>
-      </c>
-      <c r="F10" s="22">
-        <v>0</v>
-      </c>
-      <c r="G10" s="23">
+      <c r="B11" s="29"/>
+      <c r="C11" s="16">
+        <v>0</v>
+      </c>
+      <c r="D11" s="16">
+        <v>0</v>
+      </c>
+      <c r="E11" s="22">
+        <v>0</v>
+      </c>
+      <c r="F11" s="22">
+        <v>0</v>
+      </c>
+      <c r="G11" s="23">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="E3:G3"/>
+    <mergeCell ref="A11:B11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>